<commit_message>
Record QA ticket implementation and two bugs found while testing
Marks the 37 module QA tickets plus RMC-019 as done in the ticket sheet
(commits d71c702, 1f60ed2, cc82acd, f5fecaa) and adds Appendix D.1 to the
audit doc documenting two previously-unknown, pre-existing bugs surfaced
while writing the tests: teacher payment-access login is unconditionally
broken (camelCase/snake_case field mismatch between repository and
service), and translation DTO validation is partially bypassed by
class-transformer's implicit type coercion. Both predate this project's
work and are left unfixed, pinned by characterization tests instead.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ka8oy6KEy3PYBopvAdR5Cs
</commit_message>
<xml_diff>
--- a/docs/RMC-backend-audit-tickets.xlsx
+++ b/docs/RMC-backend-audit-tickets.xlsx
@@ -1988,11 +1988,19 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Logic-change analysis (this conversation)</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+          <t>Logic-change analysis (this conversation) | Implemented: commit verified directly (no code change needed)</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -4212,11 +4220,19 @@
       <c r="K54" s="4" t="inlineStr"/>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>Master table: students</t>
-        </is>
-      </c>
-      <c r="M54" s="4" t="inlineStr"/>
-      <c r="N54" s="4" t="inlineStr"/>
+          <t>Master table: students | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -4272,11 +4288,19 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Master table: teachers</t>
-        </is>
-      </c>
-      <c r="M55" s="4" t="inlineStr"/>
-      <c r="N55" s="4" t="inlineStr"/>
+          <t>Master table: teachers | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -4332,11 +4356,19 @@
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Master table: parents</t>
-        </is>
-      </c>
-      <c r="M56" s="4" t="inlineStr"/>
-      <c r="N56" s="4" t="inlineStr"/>
+          <t>Master table: parents | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -4392,11 +4424,19 @@
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>Master table: owners</t>
-        </is>
-      </c>
-      <c r="M57" s="4" t="inlineStr"/>
-      <c r="N57" s="4" t="inlineStr"/>
+          <t>Master table: owners | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -4452,11 +4492,19 @@
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>Master table: superusers</t>
-        </is>
-      </c>
-      <c r="M58" s="4" t="inlineStr"/>
-      <c r="N58" s="4" t="inlineStr"/>
+          <t>Master table: superusers | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4512,11 +4560,19 @@
       </c>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>Master table: centers</t>
-        </is>
-      </c>
-      <c r="M59" s="4" t="inlineStr"/>
-      <c r="N59" s="4" t="inlineStr"/>
+          <t>Master table: centers | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -4572,11 +4628,19 @@
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>Master table: teacherTasks</t>
-        </is>
-      </c>
-      <c r="M60" s="4" t="inlineStr"/>
-      <c r="N60" s="4" t="inlineStr"/>
+          <t>Master table: teacherTasks | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4632,11 +4696,19 @@
       </c>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>Master table: classes</t>
-        </is>
-      </c>
-      <c r="M61" s="4" t="inlineStr"/>
-      <c r="N61" s="4" t="inlineStr"/>
+          <t>Master table: classes | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -4692,11 +4764,19 @@
       </c>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>Master table: subjects</t>
-        </is>
-      </c>
-      <c r="M62" s="4" t="inlineStr"/>
-      <c r="N62" s="4" t="inlineStr"/>
+          <t>Master table: subjects | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4752,11 +4832,19 @@
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>Master table: grades</t>
-        </is>
-      </c>
-      <c r="M63" s="4" t="inlineStr"/>
-      <c r="N63" s="4" t="inlineStr"/>
+          <t>Master table: grades | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -4812,11 +4900,19 @@
       </c>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>Master table: attendance</t>
-        </is>
-      </c>
-      <c r="M64" s="4" t="inlineStr"/>
-      <c r="N64" s="4" t="inlineStr"/>
+          <t>Master table: attendance | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M64" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N64" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4872,11 +4968,19 @@
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>Master table: assignments</t>
-        </is>
-      </c>
-      <c r="M65" s="4" t="inlineStr"/>
-      <c r="N65" s="4" t="inlineStr"/>
+          <t>Master table: assignments | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M65" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -4932,11 +5036,19 @@
       </c>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>Master table: tests</t>
-        </is>
-      </c>
-      <c r="M66" s="4" t="inlineStr"/>
-      <c r="N66" s="4" t="inlineStr"/>
+          <t>Master table: tests | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -4992,11 +5104,19 @@
       </c>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>Master table: sessions</t>
-        </is>
-      </c>
-      <c r="M67" s="4" t="inlineStr"/>
-      <c r="N67" s="4" t="inlineStr"/>
+          <t>Master table: sessions | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -5052,11 +5172,19 @@
       </c>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>Master table: payments</t>
-        </is>
-      </c>
-      <c r="M68" s="4" t="inlineStr"/>
-      <c r="N68" s="4" t="inlineStr"/>
+          <t>Master table: payments | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M68" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N68" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -5112,11 +5240,19 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>Master table: payment_plans</t>
-        </is>
-      </c>
-      <c r="M69" s="4" t="inlineStr"/>
-      <c r="N69" s="4" t="inlineStr"/>
+          <t>Master table: payment_plans | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -5172,11 +5308,19 @@
       </c>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>Master table: invoices</t>
-        </is>
-      </c>
-      <c r="M70" s="4" t="inlineStr"/>
-      <c r="N70" s="4" t="inlineStr"/>
+          <t>Master table: invoices | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N70" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -5232,11 +5376,19 @@
       </c>
       <c r="L71" s="4" t="inlineStr">
         <is>
-          <t>Master table: debts</t>
-        </is>
-      </c>
-      <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" s="4" t="inlineStr"/>
+          <t>Master table: debts | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M71" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N71" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -5292,11 +5444,19 @@
       </c>
       <c r="L72" s="4" t="inlineStr">
         <is>
-          <t>Master table: discounts</t>
-        </is>
-      </c>
-      <c r="M72" s="4" t="inlineStr"/>
-      <c r="N72" s="4" t="inlineStr"/>
+          <t>Master table: discounts | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M72" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N72" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -5352,11 +5512,19 @@
       </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>Master table: refunds</t>
-        </is>
-      </c>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
+          <t>Master table: refunds | Implemented: commit 1f60ed2</t>
+        </is>
+      </c>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -5408,11 +5576,19 @@
       <c r="K74" s="4" t="inlineStr"/>
       <c r="L74" s="4" t="inlineStr">
         <is>
-          <t>Master table: salaries</t>
-        </is>
-      </c>
-      <c r="M74" s="4" t="inlineStr"/>
-      <c r="N74" s="4" t="inlineStr"/>
+          <t>Master table: salaries | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M74" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N74" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -5464,11 +5640,19 @@
       <c r="K75" s="4" t="inlineStr"/>
       <c r="L75" s="4" t="inlineStr">
         <is>
-          <t>Master table: kpis</t>
-        </is>
-      </c>
-      <c r="M75" s="4" t="inlineStr"/>
-      <c r="N75" s="4" t="inlineStr"/>
+          <t>Master table: kpis | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -5524,11 +5708,19 @@
       </c>
       <c r="L76" s="4" t="inlineStr">
         <is>
-          <t>Master table: notifications</t>
-        </is>
-      </c>
-      <c r="M76" s="4" t="inlineStr"/>
-      <c r="N76" s="4" t="inlineStr"/>
+          <t>Master table: notifications | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M76" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N76" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -5584,11 +5776,19 @@
       </c>
       <c r="L77" s="4" t="inlineStr">
         <is>
-          <t>Master table: telegram_registrations</t>
-        </is>
-      </c>
-      <c r="M77" s="4" t="inlineStr"/>
-      <c r="N77" s="4" t="inlineStr"/>
+          <t>Master table: telegram_registrations | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N77" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -5644,11 +5844,19 @@
       </c>
       <c r="L78" s="4" t="inlineStr">
         <is>
-          <t>Master table: telegram_students</t>
-        </is>
-      </c>
-      <c r="M78" s="4" t="inlineStr"/>
-      <c r="N78" s="4" t="inlineStr"/>
+          <t>Master table: telegram_students | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M78" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N78" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -5704,11 +5912,19 @@
       </c>
       <c r="L79" s="4" t="inlineStr">
         <is>
-          <t>Master table: calendar</t>
-        </is>
-      </c>
-      <c r="M79" s="4" t="inlineStr"/>
-      <c r="N79" s="4" t="inlineStr"/>
+          <t>Master table: calendar | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N79" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -5764,11 +5980,19 @@
       </c>
       <c r="L80" s="4" t="inlineStr">
         <is>
-          <t>Master table: translations</t>
-        </is>
-      </c>
-      <c r="M80" s="4" t="inlineStr"/>
-      <c r="N80" s="4" t="inlineStr"/>
+          <t>Master table: translations | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M80" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N80" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -5820,11 +6044,19 @@
       <c r="K81" s="4" t="inlineStr"/>
       <c r="L81" s="4" t="inlineStr">
         <is>
-          <t>Master table: portal</t>
-        </is>
-      </c>
-      <c r="M81" s="4" t="inlineStr"/>
-      <c r="N81" s="4" t="inlineStr"/>
+          <t>Master table: portal | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M81" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -5876,11 +6108,19 @@
       <c r="K82" s="4" t="inlineStr"/>
       <c r="L82" s="4" t="inlineStr">
         <is>
-          <t>Master table: search</t>
-        </is>
-      </c>
-      <c r="M82" s="4" t="inlineStr"/>
-      <c r="N82" s="4" t="inlineStr"/>
+          <t>Master table: search | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M82" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N82" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5936,11 +6176,19 @@
       </c>
       <c r="L83" s="4" t="inlineStr">
         <is>
-          <t>Master table: saved_filters</t>
-        </is>
-      </c>
-      <c r="M83" s="4" t="inlineStr"/>
-      <c r="N83" s="4" t="inlineStr"/>
+          <t>Master table: saved_filters | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M83" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -5996,11 +6244,19 @@
       </c>
       <c r="L84" s="4" t="inlineStr">
         <is>
-          <t>Master table: system</t>
-        </is>
-      </c>
-      <c r="M84" s="4" t="inlineStr"/>
-      <c r="N84" s="4" t="inlineStr"/>
+          <t>Master table: system | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M84" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N84" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -6056,11 +6312,19 @@
       </c>
       <c r="L85" s="4" t="inlineStr">
         <is>
-          <t>Master table: settings</t>
-        </is>
-      </c>
-      <c r="M85" s="4" t="inlineStr"/>
-      <c r="N85" s="4" t="inlineStr"/>
+          <t>Master table: settings | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -6116,11 +6380,19 @@
       </c>
       <c r="L86" s="4" t="inlineStr">
         <is>
-          <t>Master table: audit_logs</t>
-        </is>
-      </c>
-      <c r="M86" s="4" t="inlineStr"/>
-      <c r="N86" s="4" t="inlineStr"/>
+          <t>Master table: audit_logs | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M86" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N86" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -6176,11 +6448,19 @@
       </c>
       <c r="L87" s="4" t="inlineStr">
         <is>
-          <t>Master table: archive</t>
-        </is>
-      </c>
-      <c r="M87" s="4" t="inlineStr"/>
-      <c r="N87" s="4" t="inlineStr"/>
+          <t>Master table: archive | Implemented: commit d71c702</t>
+        </is>
+      </c>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N87" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -6236,11 +6516,19 @@
       </c>
       <c r="L88" s="4" t="inlineStr">
         <is>
-          <t>Master table: import_export</t>
-        </is>
-      </c>
-      <c r="M88" s="4" t="inlineStr"/>
-      <c r="N88" s="4" t="inlineStr"/>
+          <t>Master table: import_export | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M88" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N88" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -6292,11 +6580,19 @@
       <c r="K89" s="4" t="inlineStr"/>
       <c r="L89" s="4" t="inlineStr">
         <is>
-          <t>Master table: reports</t>
-        </is>
-      </c>
-      <c r="M89" s="4" t="inlineStr"/>
-      <c r="N89" s="4" t="inlineStr"/>
+          <t>Master table: reports | Implemented: commit f5fecaa</t>
+        </is>
+      </c>
+      <c r="M89" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N89" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -6352,11 +6648,19 @@
       </c>
       <c r="L90" s="4" t="inlineStr">
         <is>
-          <t>Master table: rooms</t>
-        </is>
-      </c>
-      <c r="M90" s="4" t="inlineStr"/>
-      <c r="N90" s="4" t="inlineStr"/>
+          <t>Master table: rooms | Implemented: commit cc82acd</t>
+        </is>
+      </c>
+      <c r="M90" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="N90" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N90"/>

</xml_diff>